<commit_message>
Reclasser sauce à salade, garniture bruschetta et plats préparés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01161sSjzGnJNhrD4Bz4LWVE
</commit_message>
<xml_diff>
--- a/promotions_extraites.xlsx
+++ b/promotions_extraites.xlsx
@@ -3725,11 +3725,11 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -6979,11 +6979,11 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9428,11 +9428,11 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="N202" s="2" t="n">
@@ -10136,11 +10136,11 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="N223" s="2" t="n">
@@ -11014,11 +11014,11 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="N250" s="2" t="n">

</xml_diff>

<commit_message>
Scinder 7.5 (plats préparés) et 7.6 (sauces et condiments)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01161sSjzGnJNhrD4Bz4LWVE
</commit_message>
<xml_diff>
--- a/promotions_extraites.xlsx
+++ b/promotions_extraites.xlsx
@@ -1620,11 +1620,11 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3810,11 +3810,11 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -4055,11 +4055,11 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="N79" s="2" t="n">
@@ -5245,11 +5245,11 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="N202" s="2" t="n">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="N230" s="2" t="n">
@@ -10985,11 +10985,11 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="N249" s="2" t="n">

</xml_diff>

<commit_message>
Préparations panées à base de poisson en 7.5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01161sSjzGnJNhrD4Bz4LWVE
</commit_message>
<xml_diff>
--- a/promotions_extraites.xlsx
+++ b/promotions_extraites.xlsx
@@ -6661,11 +6661,11 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -7362,11 +7362,11 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">

</xml_diff>

<commit_message>
Catégories 9 (compléments alimentaires) et 10 (condiments et ingrédients)
- 7.6 remplacée par 10.1 Sauces et condiments
- 10.2 Ingrédients bruts : levure, poudre à lever, bicarbonate, farines
- Whey protéinée en 9.1, pâtés de poisson/viande en 7.2, pâte à tarte en 7.5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01161sSjzGnJNhrD4Bz4LWVE
</commit_message>
<xml_diff>
--- a/promotions_extraites.xlsx
+++ b/promotions_extraites.xlsx
@@ -1171,12 +1171,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.2 Ingrédients bruts</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1522,12 +1522,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.2 Ingrédients bruts</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2644,12 +2644,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.2 Ingrédients bruts</t>
         </is>
       </c>
       <c r="N46" s="2" t="n">
@@ -2722,12 +2722,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>3. Produits céréaliers et pommes de terre</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>3.5 Autres</t>
+          <t>10.2 Ingrédients bruts</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2873,12 +2873,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3. Produits céréaliers et pommes de terre</t>
+          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>3.5 Autres</t>
+          <t>7.5 Plats préparés, pizzas, pâtes farcies, préparations panées</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3034,12 +3034,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3070,12 +3070,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="N56" s="2" t="n">
@@ -3101,12 +3101,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="N57" s="2" t="n">
@@ -3658,12 +3658,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5. Légumineuses, œufs, viande et autres</t>
+          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>5.3 Poisson</t>
+          <t>7.2 Snacks salés</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -3746,12 +3746,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -3793,12 +3793,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -7087,12 +7087,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>5. Légumineuses, œufs, viande et autres</t>
+          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>5.2 Charcuterie</t>
+          <t>7.2 Snacks salés</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -7278,12 +7278,12 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="N152" s="2" t="n">
@@ -9277,12 +9277,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -9324,12 +9324,12 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>3. Produits céréaliers et pommes de terre</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>3.5 Autres</t>
+          <t>10.2 Ingrédients bruts</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -13550,12 +13550,12 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="N286" s="2" t="n">
@@ -19055,12 +19055,12 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
@@ -19102,12 +19102,12 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="H405" t="inlineStr">
@@ -19196,12 +19196,12 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
@@ -19839,12 +19839,12 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>4. Produits laitiers</t>
+          <t>9. Compléments alimentaires</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>4.5 Autres</t>
+          <t>9.1 Compléments alimentaires</t>
         </is>
       </c>
       <c r="H421" t="inlineStr">
@@ -19891,12 +19891,12 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>3. Produits céréaliers et pommes de terre</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>3.5 Autres</t>
+          <t>10.2 Ingrédients bruts</t>
         </is>
       </c>
       <c r="K422" t="inlineStr">
@@ -21252,12 +21252,12 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="H452" t="inlineStr">
@@ -29345,12 +29345,12 @@
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K621" t="inlineStr">
@@ -29471,12 +29471,12 @@
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K624" t="inlineStr">
@@ -30164,12 +30164,12 @@
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K640" t="inlineStr">
@@ -33519,12 +33519,12 @@
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="K714" t="inlineStr">
@@ -33592,12 +33592,12 @@
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="N716" s="2" t="n">
@@ -34559,12 +34559,12 @@
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
+          <t>10. Condiments et ingrédients</t>
         </is>
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>7.6 Sauces et condiments</t>
+          <t>10.1 Sauces et condiments</t>
         </is>
       </c>
       <c r="N744" s="2" t="n">

</xml_diff>

<commit_message>
Tartinables salés en 7.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01161sSjzGnJNhrD4Bz4LWVE
</commit_message>
<xml_diff>
--- a/promotions_extraites.xlsx
+++ b/promotions_extraites.xlsx
@@ -30164,12 +30164,12 @@
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>10. Condiments et ingrédients</t>
+          <t>7. Boissons sucrées, sucreries, snacks salés, plats préparés et condiments</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>10.1 Sauces et condiments</t>
+          <t>7.2 Snacks salés</t>
         </is>
       </c>
       <c r="K640" t="inlineStr">

</xml_diff>